<commit_message>
add gif and updated file
</commit_message>
<xml_diff>
--- a/TEST.xlsx
+++ b/TEST.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GIT_test\Test_repository\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CE75F3B1-0651-495A-A933-0D43F7E222CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA9AFD57-5049-4876-A039-3B5F8A47C794}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{ED84DF03-3ABB-41E6-9BD8-FDA5A8B55442}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t xml:space="preserve">ID </t>
   </si>
@@ -46,6 +46,9 @@
   </si>
   <si>
     <t>E</t>
+  </si>
+  <si>
+    <t>FULL_NAME</t>
   </si>
 </sst>
 </file>
@@ -75,7 +78,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -84,71 +87,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -157,14 +105,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -479,59 +427,83 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A2A9CBA-E2FF-409E-BBBE-46FF7846A75F}">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" s="1" t="s">
+        <v>7</v>
+      </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="1">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
+      <c r="C2" s="2" t="str">
+        <f>_xlfn.IFS(B2="A", "APPLE",B2="B","BALL",B2="C", "CAT",B2="D", "DOG",B2="E", "ELEPHANT")</f>
+        <v>APPLE</v>
+      </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="1">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A3" s="2">
         <v>2</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="C3" s="2" t="str">
+        <f t="shared" ref="C3:C6" si="0">_xlfn.IFS(B3="A", "APPLE",B3="B","BALL",B3="C", "CAT",B3="D", "DOG",B3="E", "ELEPHANT")</f>
+        <v>BALL</v>
+      </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="1">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
+      <c r="C4" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>CAT</v>
+      </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A5" s="1">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A5" s="2">
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
+      <c r="C5" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>DOG</v>
+      </c>
     </row>
-    <row r="6" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A6" s="3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="s">
+      <c r="B6" s="2" t="s">
         <v>6</v>
+      </c>
+      <c r="C6" s="2" t="str">
+        <f t="shared" si="0"/>
+        <v>ELEPHANT</v>
       </c>
     </row>
   </sheetData>

</xml_diff>